<commit_message>
Write docs, test data and comments in English
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BUG-REPORT.xlsx
+++ b/docs/BUG-REPORT.xlsx
@@ -16,7 +16,7 @@
     <t>Build</t>
   </si>
   <si>
-    <t>อาการบั๊ก</t>
+    <t>Bug</t>
   </si>
   <si>
     <t>Input</t>
@@ -28,13 +28,13 @@
     <t>Actual</t>
   </si>
   <si>
-    <t>ความรุนแรง</t>
+    <t>Severity</t>
   </si>
   <si>
     <t>1</t>
   </si>
   <si>
-    <t>ไม่ตรวจสอบว่า input เป็นตัวเลข ไม่แสดงข้อความ error แต่แสดง NaN แทน</t>
+    <t>Input is not checked for numbers; shows NaN instead of an error</t>
   </si>
   <si>
     <t>Add, First = abc, Second = 3 (TC36)</t>
@@ -43,7 +43,7 @@
     <t>Error: Number 1 is not a number</t>
   </si>
   <si>
-    <t>Answer = NaN, ไม่มีข้อความ error</t>
+    <t>Answer = NaN, no error message</t>
   </si>
   <si>
     <t>Major</t>
@@ -52,7 +52,7 @@
     <t>2</t>
   </si>
   <si>
-    <t>Add กับ Concatenate ทำงานสลับกัน</t>
+    <t>Add and Concatenate are swapped</t>
   </si>
   <si>
     <t>Add, First = 2, Second = 3 (TC01)</t>
@@ -70,7 +70,7 @@
     <t>3</t>
   </si>
   <si>
-    <t>Concatenate ตรวจสอบตัวเลขเหมือนการคำนวณ ต่อข้อความที่เป็นตัวอักษรไม่ได้</t>
+    <t>Concatenate checks for numbers, so text cannot be joined</t>
   </si>
   <si>
     <t>Concatenate, First = abc, Second = def (TC27)</t>
@@ -79,13 +79,13 @@
     <t>abcdef</t>
   </si>
   <si>
-    <t>Answer ว่าง, Error: Number 1 is not a number</t>
+    <t>Answer empty, Error: Number 1 is not a number</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
-    <t>Integers only ถูกติ๊กค้างและเอาออกไม่ได้ ผลลัพธ์ทศนิยมถูกตัดทิ้งเสมอ</t>
+    <t>Integers only is always ticked and cannot be unticked, so decimals are always cut off</t>
   </si>
   <si>
     <t>Divide, First = 7, Second = 2, Integers only = No (TC21)</t>
@@ -94,16 +94,16 @@
     <t>3.5</t>
   </si>
   <si>
-    <t>ปุ่ม Clear กดไม่ได้ตอนเปิดหน้า (กดได้หลังคำนวณครั้งแรก)</t>
-  </si>
-  <si>
-    <t>เปิดหน้าแล้วกด Clear (TC44)</t>
-  </si>
-  <si>
-    <t>ปุ่ม Clear กดได้</t>
-  </si>
-  <si>
-    <t>ปุ่ม Clear ถูก disable</t>
+    <t>Clear button is disabled when the page loads and only works after the first calculation</t>
+  </si>
+  <si>
+    <t>Click Clear right after the page loads (TC44)</t>
+  </si>
+  <si>
+    <t>Clear button is enabled</t>
+  </si>
+  <si>
+    <t>Clear button is disabled</t>
   </si>
   <si>
     <t>Minor</t>
@@ -112,7 +112,7 @@
     <t>6</t>
   </si>
   <si>
-    <t>หารด้วยศูนย์แล้วไม่แสดงข้อความ error</t>
+    <t>Divide by zero shows no error</t>
   </si>
   <si>
     <t>Divide, First = 5, Second = 0 (TC25)</t>
@@ -121,22 +121,22 @@
     <t>Error: Divide by zero error!</t>
   </si>
   <si>
-    <t>Answer = Infinity, ไม่มีข้อความ error</t>
+    <t>Answer = Infinity, no error message</t>
   </si>
   <si>
     <t>7</t>
   </si>
   <si>
-    <t>ใช้ผลลัพธ์ครั้งก่อนแทนค่า First number</t>
-  </si>
-  <si>
-    <t>Add, First = 2, Second = 3 บนหน้าที่เพิ่งเปิด (TC01)</t>
+    <t>Uses the previous answer in place of First number</t>
+  </si>
+  <si>
+    <t>Add, First = 2, Second = 3 on a freshly loaded page (TC01)</t>
   </si>
   <si>
     <t>8</t>
   </si>
   <si>
-    <t>First number กับ Second number ถูกสลับกัน</t>
+    <t>First number and Second number are swapped</t>
   </si>
   <si>
     <t>Subtract, First = 5, Second = 3 (TC09)</t>
@@ -148,10 +148,10 @@
     <t>9</t>
   </si>
   <si>
-    <t>ช่อง Second number และปุ่ม Calculate หายไป คำนวณไม่ได้เลย</t>
-  </si>
-  <si>
-    <t>ไม่มีช่อง Second number และปุ่ม Calculate ให้ใช้</t>
+    <t>Second number field and Calculate button are missing, so nothing can be calculated</t>
+  </si>
+  <si>
+    <t>No Second number field or Calculate button</t>
   </si>
 </sst>
 </file>
@@ -170,11 +170,11 @@
       <b/>
       <color rgb="FFFFFFFF"/>
       <sz val="10"/>
-      <name val="Tahoma"/>
+      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Tahoma"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="3">
@@ -569,10 +569,10 @@
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="48" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
     <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="34" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -776,6 +776,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>